<commit_message>
update breakdown and skip registry for phase3 block
</commit_message>
<xml_diff>
--- a/data/gallery_lists/rag_gellery_breakdown_master.xlsx
+++ b/data/gallery_lists/rag_gellery_breakdown_master.xlsx
@@ -3470,22 +3470,56 @@
       <c r="Z46" s="7" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="40">
-      <c r="A47" s="36" t="n"/>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-      <c r="I47" s="28" t="n"/>
-      <c r="J47" s="28" t="n"/>
-      <c r="K47" s="28" t="n"/>
-      <c r="L47" s="28" t="n"/>
-      <c r="M47" s="28" t="n"/>
+      <c r="A47" s="36" t="inlineStr">
+        <is>
+          <t>Taka Ishii Gallery</t>
+        </is>
+      </c>
+      <c r="B47" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E47" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="J47" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="28" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="L47" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" s="28" t="n">
+        <v>7</v>
+      </c>
       <c r="N47" s="29" t="n"/>
-      <c r="O47" s="29" t="n"/>
-      <c r="P47" s="29" t="n"/>
+      <c r="O47" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P47" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q47" s="29" t="n"/>
       <c r="R47" s="29" t="n"/>
       <c r="S47" s="29" t="n"/>
@@ -3498,22 +3532,56 @@
       <c r="Z47" s="7" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="40">
-      <c r="A48" s="36" t="n"/>
-      <c r="B48" s="27" t="n"/>
-      <c r="C48" s="27" t="n"/>
-      <c r="D48" s="27" t="n"/>
-      <c r="E48" s="27" t="n"/>
-      <c r="F48" s="27" t="n"/>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="27" t="n"/>
-      <c r="I48" s="28" t="n"/>
-      <c r="J48" s="28" t="n"/>
-      <c r="K48" s="28" t="n"/>
-      <c r="L48" s="28" t="n"/>
-      <c r="M48" s="28" t="n"/>
+      <c r="A48" s="36" t="inlineStr">
+        <is>
+          <t>Jhaveri Contemporary</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="C48" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="D48" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E48" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>150</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="I48" s="28" t="n">
+        <v>24</v>
+      </c>
+      <c r="J48" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K48" s="28" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="L48" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="M48" s="28" t="n">
+        <v>24</v>
+      </c>
       <c r="N48" s="29" t="n"/>
-      <c r="O48" s="29" t="n"/>
-      <c r="P48" s="29" t="n"/>
+      <c r="O48" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P48" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q48" s="29" t="n"/>
       <c r="R48" s="29" t="n"/>
       <c r="S48" s="29" t="n"/>
@@ -3526,22 +3594,56 @@
       <c r="Z48" s="7" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="40">
-      <c r="A49" s="36" t="n"/>
-      <c r="B49" s="27" t="n"/>
-      <c r="C49" s="27" t="n"/>
-      <c r="D49" s="27" t="n"/>
-      <c r="E49" s="27" t="n"/>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="28" t="n"/>
-      <c r="J49" s="28" t="n"/>
-      <c r="K49" s="28" t="n"/>
-      <c r="L49" s="28" t="n"/>
-      <c r="M49" s="28" t="n"/>
+      <c r="A49" s="36" t="inlineStr">
+        <is>
+          <t>Johyun Gallery</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="C49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="D49" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="F49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="G49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>41</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>16</v>
+      </c>
+      <c r="J49" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K49" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="L49" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="M49" s="28" t="n">
+        <v>16</v>
+      </c>
       <c r="N49" s="29" t="n"/>
-      <c r="O49" s="29" t="n"/>
-      <c r="P49" s="29" t="n"/>
+      <c r="O49" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P49" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q49" s="29" t="n"/>
       <c r="R49" s="29" t="n"/>
       <c r="S49" s="29" t="n"/>
@@ -3554,22 +3656,56 @@
       <c r="Z49" s="7" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="40">
-      <c r="A50" s="36" t="n"/>
-      <c r="B50" s="27" t="n"/>
-      <c r="C50" s="27" t="n"/>
-      <c r="D50" s="27" t="n"/>
-      <c r="E50" s="27" t="n"/>
-      <c r="F50" s="27" t="n"/>
-      <c r="G50" s="27" t="n"/>
-      <c r="H50" s="27" t="n"/>
-      <c r="I50" s="28" t="n"/>
-      <c r="J50" s="28" t="n"/>
-      <c r="K50" s="28" t="n"/>
-      <c r="L50" s="28" t="n"/>
-      <c r="M50" s="28" t="n"/>
+      <c r="A50" s="36" t="inlineStr">
+        <is>
+          <t>Kalfayan Galleries</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E50" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="J50" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="28" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="L50" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" s="28" t="n">
+        <v>7</v>
+      </c>
       <c r="N50" s="29" t="n"/>
-      <c r="O50" s="29" t="n"/>
-      <c r="P50" s="29" t="n"/>
+      <c r="O50" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P50" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q50" s="29" t="n"/>
       <c r="R50" s="29" t="n"/>
       <c r="S50" s="29" t="n"/>
@@ -3582,22 +3718,56 @@
       <c r="Z50" s="7" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="40">
-      <c r="A51" s="36" t="n"/>
-      <c r="B51" s="27" t="n"/>
-      <c r="C51" s="27" t="n"/>
-      <c r="D51" s="27" t="n"/>
-      <c r="E51" s="27" t="n"/>
-      <c r="F51" s="27" t="n"/>
-      <c r="G51" s="27" t="n"/>
-      <c r="H51" s="27" t="n"/>
-      <c r="I51" s="28" t="n"/>
-      <c r="J51" s="28" t="n"/>
-      <c r="K51" s="28" t="n"/>
-      <c r="L51" s="28" t="n"/>
-      <c r="M51" s="28" t="n"/>
+      <c r="A51" s="36" t="inlineStr">
+        <is>
+          <t>Karma</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="C51" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="D51" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E51" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="F51" s="27" t="n">
+        <v>66</v>
+      </c>
+      <c r="G51" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>24</v>
+      </c>
+      <c r="J51" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K51" s="28" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="L51" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="M51" s="28" t="n">
+        <v>24</v>
+      </c>
       <c r="N51" s="29" t="n"/>
-      <c r="O51" s="29" t="n"/>
-      <c r="P51" s="29" t="n"/>
+      <c r="O51" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P51" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q51" s="29" t="n"/>
       <c r="R51" s="29" t="n"/>
       <c r="S51" s="29" t="n"/>
@@ -22329,22 +22499,56 @@
       <c r="Z47" s="7" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="40">
-      <c r="A48" s="35" t="n"/>
-      <c r="B48" s="27" t="n"/>
-      <c r="C48" s="27" t="n"/>
-      <c r="D48" s="27" t="n"/>
-      <c r="E48" s="27" t="n"/>
-      <c r="F48" s="27" t="n"/>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="27" t="n"/>
-      <c r="I48" s="28" t="n"/>
-      <c r="J48" s="28" t="n"/>
-      <c r="K48" s="28" t="n"/>
-      <c r="L48" s="28" t="n"/>
-      <c r="M48" s="28" t="n"/>
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Turnus</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E48" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I48" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="J48" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K48" s="28" t="n">
+        <v>66.66666666666667</v>
+      </c>
+      <c r="L48" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="M48" s="28" t="n">
+        <v>12</v>
+      </c>
       <c r="N48" s="29" t="n"/>
-      <c r="O48" s="29" t="n"/>
-      <c r="P48" s="29" t="n"/>
+      <c r="O48" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P48" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q48" s="29" t="n"/>
       <c r="R48" s="29" t="n"/>
       <c r="S48" s="29" t="n"/>
@@ -22357,22 +22561,54 @@
       <c r="Z48" s="7" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="40">
-      <c r="A49" s="35" t="n"/>
-      <c r="B49" s="27" t="n"/>
-      <c r="C49" s="27" t="n"/>
+      <c r="A49" s="35" t="inlineStr">
+        <is>
+          <t>Valerie's Factory</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="D49" s="27" t="n"/>
-      <c r="E49" s="27" t="n"/>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="28" t="n"/>
-      <c r="J49" s="28" t="n"/>
-      <c r="K49" s="28" t="n"/>
-      <c r="L49" s="28" t="n"/>
-      <c r="M49" s="28" t="n"/>
+      <c r="E49" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M49" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="N49" s="29" t="n"/>
-      <c r="O49" s="29" t="n"/>
-      <c r="P49" s="29" t="n"/>
+      <c r="O49" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P49" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q49" s="29" t="n"/>
       <c r="R49" s="29" t="n"/>
       <c r="S49" s="29" t="n"/>
@@ -22385,22 +22621,56 @@
       <c r="Z49" s="7" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="40">
-      <c r="A50" s="35" t="n"/>
-      <c r="B50" s="27" t="n"/>
-      <c r="C50" s="27" t="n"/>
-      <c r="D50" s="27" t="n"/>
-      <c r="E50" s="27" t="n"/>
-      <c r="F50" s="27" t="n"/>
-      <c r="G50" s="27" t="n"/>
-      <c r="H50" s="27" t="n"/>
-      <c r="I50" s="28" t="n"/>
-      <c r="J50" s="28" t="n"/>
-      <c r="K50" s="28" t="n"/>
-      <c r="L50" s="28" t="n"/>
-      <c r="M50" s="28" t="n"/>
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Vanguard Gallery</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="C50" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E50" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>156</v>
+      </c>
+      <c r="G50" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="J50" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K50" s="28" t="n">
+        <v>88.88888888888889</v>
+      </c>
+      <c r="L50" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="M50" s="28" t="n">
+        <v>9</v>
+      </c>
       <c r="N50" s="29" t="n"/>
-      <c r="O50" s="29" t="n"/>
-      <c r="P50" s="29" t="n"/>
+      <c r="O50" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P50" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q50" s="29" t="n"/>
       <c r="R50" s="29" t="n"/>
       <c r="S50" s="29" t="n"/>
@@ -22413,22 +22683,56 @@
       <c r="Z50" s="7" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="40">
-      <c r="A51" s="35" t="n"/>
-      <c r="B51" s="27" t="n"/>
-      <c r="C51" s="27" t="n"/>
-      <c r="D51" s="27" t="n"/>
-      <c r="E51" s="27" t="n"/>
-      <c r="F51" s="27" t="n"/>
-      <c r="G51" s="27" t="n"/>
-      <c r="H51" s="27" t="n"/>
-      <c r="I51" s="28" t="n"/>
-      <c r="J51" s="28" t="n"/>
-      <c r="K51" s="28" t="n"/>
-      <c r="L51" s="28" t="n"/>
-      <c r="M51" s="28" t="n"/>
+      <c r="A51" s="35" t="inlineStr">
+        <is>
+          <t>Voloshyn Gallery</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="C51" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="D51" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E51" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="F51" s="27" t="n">
+        <v>75</v>
+      </c>
+      <c r="G51" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="J51" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" s="28" t="n">
+        <v>75</v>
+      </c>
+      <c r="L51" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="M51" s="28" t="n">
+        <v>4</v>
+      </c>
       <c r="N51" s="29" t="n"/>
-      <c r="O51" s="29" t="n"/>
-      <c r="P51" s="29" t="n"/>
+      <c r="O51" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P51" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q51" s="29" t="n"/>
       <c r="R51" s="29" t="n"/>
       <c r="S51" s="29" t="n"/>
@@ -22441,22 +22745,56 @@
       <c r="Z51" s="7" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="40">
-      <c r="A52" s="35" t="n"/>
-      <c r="B52" s="27" t="n"/>
-      <c r="C52" s="27" t="n"/>
-      <c r="D52" s="27" t="n"/>
-      <c r="E52" s="27" t="n"/>
-      <c r="F52" s="27" t="n"/>
-      <c r="G52" s="27" t="n"/>
-      <c r="H52" s="27" t="n"/>
-      <c r="I52" s="28" t="n"/>
-      <c r="J52" s="28" t="n"/>
-      <c r="K52" s="28" t="n"/>
-      <c r="L52" s="28" t="n"/>
-      <c r="M52" s="28" t="n"/>
+      <c r="A52" s="35" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="B52" s="27" t="n">
+        <v>70</v>
+      </c>
+      <c r="C52" s="27" t="n">
+        <v>70</v>
+      </c>
+      <c r="D52" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E52" s="27" t="n">
+        <v>70</v>
+      </c>
+      <c r="F52" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="27" t="n">
+        <v>70</v>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>70</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>31</v>
+      </c>
+      <c r="J52" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="28" t="n">
+        <v>31</v>
+      </c>
       <c r="N52" s="29" t="n"/>
-      <c r="O52" s="29" t="n"/>
-      <c r="P52" s="29" t="n"/>
+      <c r="O52" s="41" t="n">
+        <v>46144</v>
+      </c>
+      <c r="P52" s="29" t="inlineStr">
+        <is>
+          <t>TASK_PHASE3_BLOCK6_XLSX_UPDATE_20260502T000000Z</t>
+        </is>
+      </c>
       <c r="Q52" s="29" t="n"/>
       <c r="R52" s="29" t="n"/>
       <c r="S52" s="29" t="n"/>

</xml_diff>